<commit_message>
Update all BOMs with new Pushernut URLs and new power connectors.
</commit_message>
<xml_diff>
--- a/Modules/AxB/AxB_BOM.xlsx
+++ b/Modules/AxB/AxB_BOM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\My-Dev\Modular Synth\Avalon Harmonics\AxB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3790C51B-51F4-4E0A-9D01-8820E3B6E0B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{623FE8AE-A101-4A84-A44F-2CC0D485C0DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM" sheetId="1" r:id="rId1"/>
@@ -164,15 +164,9 @@
     <t>Pushernut</t>
   </si>
   <si>
-    <t>https://pushermanproductions.com/product/black-smooth-edge-jack-nuts-pack-of-25/</t>
-  </si>
-  <si>
     <t>Gold</t>
   </si>
   <si>
-    <t>https://pushermanproductions.com/product/pushernuts-gold-smooth-edge-jack-nuts-pack-of-25/</t>
-  </si>
-  <si>
     <t>Potentiometer Knob</t>
   </si>
   <si>
@@ -742,9 +736,6 @@
     <t>https://www.tme.eu/de/en/details/zl201-40g/pin-headers/connfly/ds1021-1-40sf11-b/</t>
   </si>
   <si>
-    <t>https://www.tme.eu/de/en/details/zl202-80g/pin-headers/connfly/ds1021-2-40sf11/</t>
-  </si>
-  <si>
     <t>https://www.buerklin.com/en/p/quadrios/wirewound-resistors/22p046/73P0034/</t>
   </si>
   <si>
@@ -776,6 +767,15 @@
   </si>
   <si>
     <t>LED 3mm Dome Bicolor</t>
+  </si>
+  <si>
+    <t>https://www.tme.eu/de/en/details/zl202-10g/pin-headers/connfly/ds1021-2-5sf11-b/</t>
+  </si>
+  <si>
+    <t>https://pushermanproductions.com/products/pushernuts-round-mini-jack-nuts-pack-of-25?variant=57164621578504</t>
+  </si>
+  <si>
+    <t>https://pushermanproductions.com/products/pushernuts-round-mini-jack-nuts-pack-of-25?variant=57166910816520</t>
   </si>
 </sst>
 </file>
@@ -1686,7 +1686,7 @@
   <sheetData>
     <row r="1" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
@@ -1710,7 +1710,7 @@
       </c>
       <c r="G2" s="1"/>
       <c r="J2" s="1" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
@@ -1721,16 +1721,16 @@
         <v>15</v>
       </c>
       <c r="C3" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="D3" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="E3" t="s">
         <v>21</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="J3" s="2" t="s">
         <v>32</v>
@@ -1741,10 +1741,10 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C4" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="D4" t="s">
         <v>14</v>
@@ -1753,7 +1753,7 @@
         <v>21</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="J4" s="2" t="s">
         <v>32</v>
@@ -1764,19 +1764,19 @@
         <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C5" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="D5" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E5" t="s">
         <v>21</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="J5" s="2" t="s">
         <v>32</v>
@@ -1790,16 +1790,16 @@
         <v>13</v>
       </c>
       <c r="C6" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="D6" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="E6" t="s">
         <v>21</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="J6" s="2" t="s">
         <v>32</v>
@@ -1810,22 +1810,22 @@
         <v>1</v>
       </c>
       <c r="B7" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C7" t="s">
+        <v>67</v>
+      </c>
+      <c r="D7" t="s">
+        <v>71</v>
+      </c>
+      <c r="E7" t="s">
+        <v>92</v>
+      </c>
+      <c r="F7" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="D7" t="s">
-        <v>73</v>
-      </c>
-      <c r="E7" t="s">
-        <v>94</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>71</v>
-      </c>
       <c r="J7" s="2" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
@@ -1836,19 +1836,19 @@
         <v>13</v>
       </c>
       <c r="C8" t="s">
+        <v>67</v>
+      </c>
+      <c r="D8" t="s">
+        <v>70</v>
+      </c>
+      <c r="E8" t="s">
+        <v>92</v>
+      </c>
+      <c r="F8" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="D8" t="s">
-        <v>72</v>
-      </c>
-      <c r="E8" t="s">
-        <v>94</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>71</v>
-      </c>
       <c r="J8" s="2" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
@@ -1856,22 +1856,22 @@
         <v>2</v>
       </c>
       <c r="B9" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C9" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D9" t="s">
         <v>8</v>
       </c>
       <c r="E9" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="J9" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
@@ -1882,19 +1882,19 @@
         <v>7</v>
       </c>
       <c r="C10" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D10" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="E10" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="J10" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
@@ -1905,19 +1905,19 @@
         <v>5</v>
       </c>
       <c r="C11" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D11" t="s">
         <v>6</v>
       </c>
       <c r="E11" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="J11" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
@@ -1937,10 +1937,10 @@
         <v>29</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="J12" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
@@ -1960,10 +1960,10 @@
         <v>30</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="J13" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
@@ -1977,13 +1977,13 @@
         <v>27</v>
       </c>
       <c r="D14" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="E14" t="s">
         <v>28</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="J14" s="2" t="s">
         <v>33</v>
@@ -2000,16 +2000,16 @@
         <v>24</v>
       </c>
       <c r="D15" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="E15" t="s">
         <v>25</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="J15" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
@@ -2017,22 +2017,22 @@
         <v>1</v>
       </c>
       <c r="B16" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C16" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="D16" t="s">
+        <v>77</v>
+      </c>
+      <c r="E16" t="s">
         <v>79</v>
       </c>
-      <c r="E16" t="s">
-        <v>81</v>
-      </c>
       <c r="F16" s="2" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="J16" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
@@ -2040,22 +2040,22 @@
         <v>2</v>
       </c>
       <c r="B17" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C17" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="E17" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="F17" s="2" t="s">
         <v>34</v>
       </c>
       <c r="J17" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
@@ -2066,19 +2066,19 @@
         <v>20</v>
       </c>
       <c r="C18" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="E18" t="s">
         <v>19</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="J18" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
@@ -2086,22 +2086,22 @@
         <v>2</v>
       </c>
       <c r="B19" t="s">
+        <v>85</v>
+      </c>
+      <c r="C19" t="s">
+        <v>88</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="E19" t="s">
+        <v>86</v>
+      </c>
+      <c r="F19" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="C19" t="s">
-        <v>90</v>
-      </c>
-      <c r="D19" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="E19" t="s">
-        <v>88</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>89</v>
-      </c>
       <c r="J19" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
@@ -2109,13 +2109,13 @@
         <v>3</v>
       </c>
       <c r="B20" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C20" t="s">
         <v>35</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="E20" t="s">
         <v>26</v>
@@ -2124,7 +2124,7 @@
         <v>36</v>
       </c>
       <c r="J20" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
@@ -2132,22 +2132,22 @@
         <v>2</v>
       </c>
       <c r="B21" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C21" t="s">
         <v>37</v>
       </c>
       <c r="D21" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="E21" t="s">
         <v>18</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="J21" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
@@ -2161,16 +2161,16 @@
         <v>37</v>
       </c>
       <c r="D22" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E22" t="s">
         <v>18</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="J22" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
@@ -2178,22 +2178,22 @@
         <v>2</v>
       </c>
       <c r="B23" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C23" t="s">
         <v>38</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="E23" t="s">
         <v>18</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="J23" s="2" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
@@ -2207,16 +2207,16 @@
         <v>38</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="E24" t="s">
         <v>18</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="J24" s="2" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
@@ -2236,10 +2236,10 @@
         <v>18</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>120</v>
+        <v>129</v>
       </c>
       <c r="J25" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
@@ -2247,19 +2247,19 @@
         <v>1</v>
       </c>
       <c r="B27" t="s">
+        <v>49</v>
+      </c>
+      <c r="C27" t="s">
+        <v>50</v>
+      </c>
+      <c r="E27" t="s">
         <v>51</v>
       </c>
-      <c r="C27" t="s">
+      <c r="F27" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="E27" t="s">
-        <v>53</v>
-      </c>
-      <c r="F27" s="2" t="s">
-        <v>54</v>
-      </c>
       <c r="J27" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
@@ -2267,19 +2267,19 @@
         <v>1</v>
       </c>
       <c r="B28" t="s">
+        <v>54</v>
+      </c>
+      <c r="C28" t="s">
+        <v>55</v>
+      </c>
+      <c r="E28" t="s">
         <v>56</v>
       </c>
-      <c r="C28" t="s">
-        <v>57</v>
-      </c>
-      <c r="E28" t="s">
-        <v>58</v>
-      </c>
       <c r="F28" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="J28" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
@@ -2287,19 +2287,19 @@
         <v>1</v>
       </c>
       <c r="B29" t="s">
+        <v>57</v>
+      </c>
+      <c r="C29" t="s">
+        <v>60</v>
+      </c>
+      <c r="E29" t="s">
         <v>59</v>
       </c>
-      <c r="C29" t="s">
-        <v>62</v>
-      </c>
-      <c r="E29" t="s">
-        <v>61</v>
-      </c>
       <c r="F29" s="2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="J29" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
@@ -2313,13 +2313,13 @@
         <v>42</v>
       </c>
       <c r="E31" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>43</v>
+        <v>130</v>
       </c>
       <c r="J31" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
@@ -2327,19 +2327,19 @@
         <v>1</v>
       </c>
       <c r="B32" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C32" t="s">
         <v>42</v>
       </c>
       <c r="E32" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>45</v>
+        <v>131</v>
       </c>
       <c r="J32" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
@@ -2350,16 +2350,16 @@
         <v>41</v>
       </c>
       <c r="C33" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E33" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="J33" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
@@ -2367,34 +2367,34 @@
         <v>2</v>
       </c>
       <c r="B34" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C34" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="E34" t="s">
+        <v>44</v>
+      </c>
+      <c r="F34" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="F34" s="2" t="s">
-        <v>48</v>
-      </c>
       <c r="J34" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B36" s="4" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B38" s="3" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B39" s="3" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
   </sheetData>
@@ -2405,39 +2405,39 @@
     <hyperlink ref="F27" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
     <hyperlink ref="F28" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
     <hyperlink ref="F29" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
-    <hyperlink ref="F31" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
-    <hyperlink ref="F32" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
-    <hyperlink ref="J23" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
-    <hyperlink ref="F21" r:id="rId10" xr:uid="{8471C66D-2803-4E39-A4C9-56382FB4FA7C}"/>
-    <hyperlink ref="F25" r:id="rId11" xr:uid="{6ABC6086-4872-4A5E-A074-AF133E043F03}"/>
-    <hyperlink ref="F7" r:id="rId12" xr:uid="{0078F1D0-2252-4276-B4FA-F7758611CB55}"/>
-    <hyperlink ref="F8" r:id="rId13" xr:uid="{C63AEC0D-8CBC-4750-A708-A0BDA2E3A104}"/>
-    <hyperlink ref="F16" r:id="rId14" xr:uid="{850880ED-5B0D-4785-BD00-D263FDB1367B}"/>
-    <hyperlink ref="F17" r:id="rId15" xr:uid="{53562666-7339-4495-85C8-BCFF4A8BDBAF}"/>
-    <hyperlink ref="F22" r:id="rId16" xr:uid="{70623DF7-AD80-49BE-8BCF-99E43397C3C6}"/>
-    <hyperlink ref="J24" r:id="rId17" xr:uid="{10E960AF-C6C6-47C3-9E72-05533B5ED5AD}"/>
-    <hyperlink ref="F19" r:id="rId18" xr:uid="{362C4AFE-495E-47D3-8980-A94395D8849C}"/>
-    <hyperlink ref="J3" r:id="rId19" xr:uid="{9E0ED9E0-C3A3-4348-BB6F-5C429B9E61E7}"/>
-    <hyperlink ref="J6" r:id="rId20" xr:uid="{AC848EF4-7FAB-4E48-AF09-F798B5BC950A}"/>
-    <hyperlink ref="J4" r:id="rId21" xr:uid="{238CA172-A99C-46CD-9FBB-BE7CBE8D9023}"/>
-    <hyperlink ref="J5" r:id="rId22" xr:uid="{7C381042-415D-491B-ACA4-70B1B604E6FF}"/>
-    <hyperlink ref="F33" r:id="rId23" xr:uid="{5285EE03-FF15-4800-B4FB-C302200D43C4}"/>
-    <hyperlink ref="J14" r:id="rId24" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
-    <hyperlink ref="F15" r:id="rId25" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
-    <hyperlink ref="F13" r:id="rId26" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
-    <hyperlink ref="F12" r:id="rId27" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
-    <hyperlink ref="F11" r:id="rId28" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="F10" r:id="rId29" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="F9" r:id="rId30" xr:uid="{1D4215ED-E169-427E-90FC-04FAE5A9B71D}"/>
-    <hyperlink ref="J7" r:id="rId31" xr:uid="{D56F3FC4-21F0-446F-A842-9A94AA04813F}"/>
-    <hyperlink ref="J8" r:id="rId32" xr:uid="{8C810300-BA98-4ED0-8B65-62815602E020}"/>
-    <hyperlink ref="F3" r:id="rId33" xr:uid="{977127FB-AC67-46C8-B0B1-0501C19A549A}"/>
-    <hyperlink ref="F4" r:id="rId34" xr:uid="{359AC861-5C21-4BF5-8FAD-ACC8E938C8D6}"/>
-    <hyperlink ref="F5" r:id="rId35" xr:uid="{3911DD1D-F5E3-40DF-975F-85923B0A46A2}"/>
-    <hyperlink ref="F6" r:id="rId36" xr:uid="{D2EB87A2-04E8-48FC-B49C-94AC093B082C}"/>
-    <hyperlink ref="F24" r:id="rId37" xr:uid="{5649177F-DDA8-4B6A-B3A4-79E4FAFB8310}"/>
-    <hyperlink ref="F23" r:id="rId38" xr:uid="{B5142C91-0B17-4672-B1DD-9DF602826583}"/>
-    <hyperlink ref="F14" r:id="rId39" xr:uid="{54A5E477-5B48-4EAE-A009-A3E26DFEBCB0}"/>
+    <hyperlink ref="J23" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
+    <hyperlink ref="F21" r:id="rId8" xr:uid="{8471C66D-2803-4E39-A4C9-56382FB4FA7C}"/>
+    <hyperlink ref="F7" r:id="rId9" xr:uid="{0078F1D0-2252-4276-B4FA-F7758611CB55}"/>
+    <hyperlink ref="F8" r:id="rId10" xr:uid="{C63AEC0D-8CBC-4750-A708-A0BDA2E3A104}"/>
+    <hyperlink ref="F16" r:id="rId11" xr:uid="{850880ED-5B0D-4785-BD00-D263FDB1367B}"/>
+    <hyperlink ref="F17" r:id="rId12" xr:uid="{53562666-7339-4495-85C8-BCFF4A8BDBAF}"/>
+    <hyperlink ref="F22" r:id="rId13" xr:uid="{70623DF7-AD80-49BE-8BCF-99E43397C3C6}"/>
+    <hyperlink ref="J24" r:id="rId14" xr:uid="{10E960AF-C6C6-47C3-9E72-05533B5ED5AD}"/>
+    <hyperlink ref="F19" r:id="rId15" xr:uid="{362C4AFE-495E-47D3-8980-A94395D8849C}"/>
+    <hyperlink ref="J3" r:id="rId16" xr:uid="{9E0ED9E0-C3A3-4348-BB6F-5C429B9E61E7}"/>
+    <hyperlink ref="J6" r:id="rId17" xr:uid="{AC848EF4-7FAB-4E48-AF09-F798B5BC950A}"/>
+    <hyperlink ref="J4" r:id="rId18" xr:uid="{238CA172-A99C-46CD-9FBB-BE7CBE8D9023}"/>
+    <hyperlink ref="J5" r:id="rId19" xr:uid="{7C381042-415D-491B-ACA4-70B1B604E6FF}"/>
+    <hyperlink ref="F33" r:id="rId20" xr:uid="{5285EE03-FF15-4800-B4FB-C302200D43C4}"/>
+    <hyperlink ref="J14" r:id="rId21" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="F15" r:id="rId22" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="F13" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="F12" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="F11" r:id="rId25" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="F10" r:id="rId26" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="F9" r:id="rId27" xr:uid="{1D4215ED-E169-427E-90FC-04FAE5A9B71D}"/>
+    <hyperlink ref="J7" r:id="rId28" xr:uid="{D56F3FC4-21F0-446F-A842-9A94AA04813F}"/>
+    <hyperlink ref="J8" r:id="rId29" xr:uid="{8C810300-BA98-4ED0-8B65-62815602E020}"/>
+    <hyperlink ref="F3" r:id="rId30" xr:uid="{977127FB-AC67-46C8-B0B1-0501C19A549A}"/>
+    <hyperlink ref="F4" r:id="rId31" xr:uid="{359AC861-5C21-4BF5-8FAD-ACC8E938C8D6}"/>
+    <hyperlink ref="F5" r:id="rId32" xr:uid="{3911DD1D-F5E3-40DF-975F-85923B0A46A2}"/>
+    <hyperlink ref="F6" r:id="rId33" xr:uid="{D2EB87A2-04E8-48FC-B49C-94AC093B082C}"/>
+    <hyperlink ref="F24" r:id="rId34" xr:uid="{5649177F-DDA8-4B6A-B3A4-79E4FAFB8310}"/>
+    <hyperlink ref="F23" r:id="rId35" xr:uid="{B5142C91-0B17-4672-B1DD-9DF602826583}"/>
+    <hyperlink ref="F14" r:id="rId36" xr:uid="{54A5E477-5B48-4EAE-A009-A3E26DFEBCB0}"/>
+    <hyperlink ref="F25" r:id="rId37" xr:uid="{C2724BD2-B61D-4845-9542-C04284F3E479}"/>
+    <hyperlink ref="F31" r:id="rId38" xr:uid="{5E88ED4F-6CC6-4087-AFA9-6DE2D871282C}"/>
+    <hyperlink ref="F32" r:id="rId39" xr:uid="{33267A49-D562-42AD-AC1C-905BC558F3EF}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId40"/>

</xml_diff>